<commit_message>
Populate employees from EOBs; add NPI & cutoff
Change employees workbook flow to read directly from reconciled EOB visits (EobVisit) instead of the schedule. Add employee -> PERF PROV NPI mapping (employee_npi.example.json / employee_npi.local.json / Streamlit secrets) and derive EMPLOYEE_APPEND_SHEETS from that mapping; Marcia is fill-only. Introduce an optional service-date cutoff applied to the reconciled visit set before consumers run. Refactor remit/config.py to generalise local/secrets map loaders. Update employees logic, previews, and Streamlit UI to show EOB NPI and cutoff, add tests and fixtures (including a fourth remittance PDF and fixtures script), and update README/CHANGELOG. Misc: various test and fixture updates, audit/stamping and dedupe behavior preserved.
</commit_message>
<xml_diff>
--- a/tests/fixtures/AMSMC_employees_sample.xlsx
+++ b/tests/fixtures/AMSMC_employees_sample.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -549,6 +549,30 @@
       <c r="D5" t="inlineStr">
         <is>
           <t>01/05/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Ravensworth, Cecily</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>06/02/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Beaumont, Sylvie</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>06/10/2026</t>
         </is>
       </c>
     </row>
@@ -563,7 +587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -632,6 +656,30 @@
       <c r="D2" t="inlineStr">
         <is>
           <t>03/04/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Whitfield, Harold</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>06/05/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Whitfield, Harold</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>06/11/2026</t>
         </is>
       </c>
     </row>
@@ -646,7 +694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -724,6 +772,30 @@
       <c r="D4" t="inlineStr">
         <is>
           <t>04/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Nakamura, Hiroshi</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>06/03/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Beaumont, Sylvie</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>06/10/2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 835 DB source and two-sheet HPSM handling
The app now reads remittances from the structured 835 SQLite source instead of PDFs, filtering to Noridian and HPSM and aggregating each payer separately. It adds a second schedule sheet (`2026 Medical`), routes new visits by payer, writes HPSM CARC 23 crossover amounts to the Medicare row's `Co-pays Paid`, and keeps the legacy PDF path available behind `REMIT_SOURCE_SCOPE` for one-off use.

The change also adds local-only DB safeguards, synthetic 835 fixtures/tests, and employee-tab copay routing so crossover payments land in the correct copay column without double-counting primary payments.
</commit_message>
<xml_diff>
--- a/tests/fixtures/AMSMC_employees_sample.xlsx
+++ b/tests/fixtures/AMSMC_employees_sample.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -573,6 +573,18 @@
       <c r="D7" t="inlineStr">
         <is>
           <t>06/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Ashgrove, Petra</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>07/06/2026</t>
         </is>
       </c>
     </row>

</xml_diff>